<commit_message>
CMBT.OL CR:c|low|missing. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/CMBT.OL.xlsx
+++ b/data/obx_xlsx/CMBT.OL.xlsx
@@ -3075,9 +3075,7 @@
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
       <c r="N31" s="15"/>
-      <c r="O31" s="16">
-        <v>142.72</v>
-      </c>
+      <c r="O31" s="16"/>
       <c r="P31" s="15"/>
       <c r="Q31" s="15"/>
       <c r="R31" s="15"/>
@@ -3149,9 +3147,6 @@
         <v>0.0</v>
       </c>
       <c r="S32" s="15"/>
-      <c r="T32" s="15"/>
-      <c r="U32" s="15"/>
-      <c r="V32" s="15"/>
       <c r="W32" s="15"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
@@ -3408,11 +3403,21 @@
       <c r="N38" s="16">
         <v>159.67</v>
       </c>
-      <c r="O38" s="15"/>
-      <c r="P38" s="15"/>
-      <c r="Q38" s="15"/>
-      <c r="R38" s="15"/>
-      <c r="S38" s="15"/>
+      <c r="O38" s="22">
+        <v>91.48</v>
+      </c>
+      <c r="P38" s="22">
+        <v>87.29</v>
+      </c>
+      <c r="Q38" s="22">
+        <v>95.71</v>
+      </c>
+      <c r="R38" s="22">
+        <v>94.35</v>
+      </c>
+      <c r="S38" s="16">
+        <v>101.07</v>
+      </c>
       <c r="T38" s="16">
         <v>120.53</v>
       </c>

</xml_diff>